<commit_message>
Updating QA Access data and associated scripts for updated run of QA
</commit_message>
<xml_diff>
--- a/data/2b_pm_nh3_voc/static_tables/qa/2022/eGRID2022_pmemissions_state.xlsx
+++ b/data/2b_pm_nh3_voc/static_tables/qa/2022/eGRID2022_pmemissions_state.xlsx
@@ -8,10 +8,9 @@
   </bookViews>
   <sheets>
     <sheet sheetId="1" r:id="rId1" name="State_file_latest_NEI_yr_with_P"/>
-    <sheet r:id="rId4" name="State_file_latest_NEI_yr_with_1" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="State_file_latest_NEI_yr_with_PM">'State_file_latest_NEI_yr_with_1'!$A$1:$D$53</definedName>
+    <definedName name="State_file_latest_NEI_yr_with_PM">'State_file_latest_NEI_yr_with_P'!$A$1:$D$53</definedName>
   </definedNames>
   <calcPr calcId="125725" fullCalcOnLoad="true"/>
 </workbook>
@@ -376,13 +375,13 @@
         </is>
       </c>
       <c r="B2" s="0">
-        <v>6595817.773</v>
+        <v>6694128.234</v>
       </c>
       <c r="C2" s="0">
-        <v>1151.2667003613</v>
+        <v>1183.97349245646</v>
       </c>
       <c r="D2" s="0">
-        <v>0.349089905143836</v>
+        <v>0.353734930395556</v>
       </c>
     </row>
     <row outlineLevel="0" r="3">
@@ -392,13 +391,13 @@
         </is>
       </c>
       <c r="B3" s="0">
-        <v>142731860.61</v>
+        <v>144788892.892</v>
       </c>
       <c r="C3" s="0">
-        <v>1550.4332004584</v>
+        <v>1940.07988943241</v>
       </c>
       <c r="D3" s="0">
-        <v>2.17251172069395E-02</v>
+        <v>2.67987391944428E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="4">
@@ -408,13 +407,13 @@
         </is>
       </c>
       <c r="B4" s="0">
-        <v>61100068.005</v>
+        <v>65905029.856</v>
       </c>
       <c r="C4" s="0">
-        <v>2153.93349483041</v>
+        <v>2484.18914916171</v>
       </c>
       <c r="D4" s="0">
-        <v>7.05051095738272E-02</v>
+        <v>7.53869364626516E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="5">
@@ -424,13 +423,13 @@
         </is>
       </c>
       <c r="B5" s="0">
-        <v>108500973.376</v>
+        <v>104698773.165</v>
       </c>
       <c r="C5" s="0">
-        <v>1833.87099669745</v>
+        <v>2033.02842595787</v>
       </c>
       <c r="D5" s="0">
-        <v>3.38037704112081E-02</v>
+        <v>3.88357640591246E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="6">
@@ -440,13 +439,13 @@
         </is>
       </c>
       <c r="B6" s="0">
-        <v>196943760.108</v>
+        <v>203256382.497</v>
       </c>
       <c r="C6" s="0">
-        <v>2001.06587330128</v>
+        <v>3495.27080754069</v>
       </c>
       <c r="D6" s="0">
-        <v>2.03211909044891E-02</v>
+        <v>3.43927286769682E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="7">
@@ -456,13 +455,13 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>56832574.334</v>
+        <v>58012255.357</v>
       </c>
       <c r="C7" s="0">
-        <v>1046.97770549756</v>
+        <v>1270.69109002107</v>
       </c>
       <c r="D7" s="0">
-        <v>3.68442822718031E-02</v>
+        <v>4.38076776088571E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="8">
@@ -472,13 +471,13 @@
         </is>
       </c>
       <c r="B8" s="0">
-        <v>44079943.539</v>
+        <v>42761369.034</v>
       </c>
       <c r="C8" s="0">
-        <v>333.697209912129</v>
+        <v>331.922671179937</v>
       </c>
       <c r="D8" s="0">
-        <v>1.51405461586805E-02</v>
+        <v>1.55244174205939E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="9">
@@ -488,13 +487,13 @@
         </is>
       </c>
       <c r="B9" s="0">
-        <v>184480.001</v>
+        <v>160237.001</v>
       </c>
       <c r="C9" s="0">
-        <v>8.76841384551192</v>
+        <v>7.9055459044218</v>
       </c>
       <c r="D9" s="0">
-        <v>9.50608607760353E-02</v>
+        <v>9.86731635650345E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="10">
@@ -504,13 +503,13 @@
         </is>
       </c>
       <c r="B10" s="0">
-        <v>4305126</v>
+        <v>5308370</v>
       </c>
       <c r="C10" s="0">
-        <v>197.499918117322</v>
+        <v>250.879158350828</v>
       </c>
       <c r="D10" s="0">
-        <v>0.091751051243249</v>
+        <v>9.45221069182547E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="11">
@@ -520,13 +519,13 @@
         </is>
       </c>
       <c r="B11" s="0">
-        <v>246185265.397</v>
+        <v>257955504.155</v>
       </c>
       <c r="C11" s="0">
-        <v>8180.86408602075</v>
+        <v>8169.759739289</v>
       </c>
       <c r="D11" s="0">
-        <v>6.64610375672015E-02</v>
+        <v>6.33423951626941E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="12">
@@ -536,13 +535,13 @@
         </is>
       </c>
       <c r="B12" s="0">
-        <v>124199775.463</v>
+        <v>126484632.485</v>
       </c>
       <c r="C12" s="0">
-        <v>1684.61377838299</v>
+        <v>2862.14913314853</v>
       </c>
       <c r="D12" s="0">
-        <v>2.71274850876819E-02</v>
+        <v>4.52568676038641E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="13">
@@ -552,13 +551,13 @@
         </is>
       </c>
       <c r="B13" s="0">
-        <v>9180590.002</v>
+        <v>9304192.004</v>
       </c>
       <c r="C13" s="0">
-        <v>3082.09128129626</v>
+        <v>2863.11047610233</v>
       </c>
       <c r="D13" s="0">
-        <v>0.671436428513816</v>
+        <v>0.615445269158555</v>
       </c>
     </row>
     <row outlineLevel="0" r="14">
@@ -568,13 +567,13 @@
         </is>
       </c>
       <c r="B14" s="0">
-        <v>67198724.482</v>
+        <v>72909386.062</v>
       </c>
       <c r="C14" s="0">
-        <v>1413.89546527555</v>
+        <v>1322.48058061623</v>
       </c>
       <c r="D14" s="0">
-        <v>4.20810209174218E-02</v>
+        <v>3.62773753023139E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="15">
@@ -584,13 +583,13 @@
         </is>
       </c>
       <c r="B15" s="0">
-        <v>16834399.801</v>
+        <v>16278410.189</v>
       </c>
       <c r="C15" s="0">
-        <v>140.985313932199</v>
+        <v>149.872489678535</v>
       </c>
       <c r="D15" s="0">
-        <v>0.016749669201016</v>
+        <v>1.84136519400168E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="16">
@@ -600,13 +599,13 @@
         </is>
       </c>
       <c r="B16" s="0">
-        <v>181296445.222</v>
+        <v>185197549.577</v>
       </c>
       <c r="C16" s="0">
-        <v>3637.24571571342</v>
+        <v>1949.41923545194</v>
       </c>
       <c r="D16" s="0">
-        <v>4.01248431678797E-02</v>
+        <v>2.10523221274202E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="17">
@@ -616,13 +615,13 @@
         </is>
       </c>
       <c r="B17" s="0">
-        <v>94126667.181</v>
+        <v>98022168.549</v>
       </c>
       <c r="C17" s="0">
-        <v>5619.0471417222</v>
+        <v>5230.59915954845</v>
       </c>
       <c r="D17" s="0">
-        <v>0.119393309250334</v>
+        <v>0.106722779897156</v>
       </c>
     </row>
     <row outlineLevel="0" r="18">
@@ -632,13 +631,13 @@
         </is>
       </c>
       <c r="B18" s="0">
-        <v>56573059.816</v>
+        <v>62194840.58</v>
       </c>
       <c r="C18" s="0">
-        <v>1078.6961317392</v>
+        <v>1064.90544996322</v>
       </c>
       <c r="D18" s="0">
-        <v>3.81346222123245E-02</v>
+        <v>3.42441733118827E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="19">
@@ -648,13 +647,13 @@
         </is>
       </c>
       <c r="B19" s="0">
-        <v>69904814.122</v>
+        <v>69146933.093</v>
       </c>
       <c r="C19" s="0">
-        <v>19134.5726552422</v>
+        <v>3194.50009645734</v>
       </c>
       <c r="D19" s="0">
-        <v>0.547446492650649</v>
+        <v>9.23974485509244E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="20">
@@ -664,13 +663,13 @@
         </is>
       </c>
       <c r="B20" s="0">
-        <v>97167796.19</v>
+        <v>105223371.518</v>
       </c>
       <c r="C20" s="0">
-        <v>2774.64238936955</v>
+        <v>3010.29752047694</v>
       </c>
       <c r="D20" s="0">
-        <v>5.71103286925242E-02</v>
+        <v>5.72172793372618E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="21">
@@ -680,13 +679,13 @@
         </is>
       </c>
       <c r="B21" s="0">
-        <v>19429416.602</v>
+        <v>21022930.789</v>
       </c>
       <c r="C21" s="0">
-        <v>1192.17703781222</v>
+        <v>1106.48090345667</v>
       </c>
       <c r="D21" s="0">
-        <v>0.122718768374085</v>
+        <v>0.105264191235945</v>
       </c>
     </row>
     <row outlineLevel="0" r="22">
@@ -696,13 +695,13 @@
         </is>
       </c>
       <c r="B22" s="0">
-        <v>38166718.985</v>
+        <v>37134094.879</v>
       </c>
       <c r="C22" s="0">
-        <v>663.210251827304</v>
+        <v>408.052402065771</v>
       </c>
       <c r="D22" s="0">
-        <v>3.47533280022291E-02</v>
+        <v>2.19772370052586E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="23">
@@ -712,13 +711,13 @@
         </is>
       </c>
       <c r="B23" s="0">
-        <v>10900945.883</v>
+        <v>12763920.003</v>
       </c>
       <c r="C23" s="0">
-        <v>411.455398777292</v>
+        <v>691.622991673066</v>
       </c>
       <c r="D23" s="0">
-        <v>7.54898525675567E-02</v>
+        <v>0.108371564771717</v>
       </c>
     </row>
     <row outlineLevel="0" r="24">
@@ -728,13 +727,13 @@
         </is>
       </c>
       <c r="B24" s="0">
-        <v>115299089.641</v>
+        <v>116615130.596</v>
       </c>
       <c r="C24" s="0">
-        <v>2200.07506407031</v>
+        <v>3355.34714861007</v>
       </c>
       <c r="D24" s="0">
-        <v>3.81629216834332E-02</v>
+        <v>5.75456569222444E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="25">
@@ -744,13 +743,13 @@
         </is>
       </c>
       <c r="B25" s="0">
-        <v>59157704.839</v>
+        <v>58966891.046</v>
       </c>
       <c r="C25" s="0">
-        <v>908.370636151082</v>
+        <v>1041.80325738326</v>
       </c>
       <c r="D25" s="0">
-        <v>3.07101378805431E-02</v>
+        <v>3.53351936621706E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="26">
@@ -760,13 +759,13 @@
         </is>
       </c>
       <c r="B26" s="0">
-        <v>76941409.993</v>
+        <v>79361031.625</v>
       </c>
       <c r="C26" s="0">
-        <v>3864.05408992328</v>
+        <v>3677.24494527519</v>
       </c>
       <c r="D26" s="0">
-        <v>0.100441468132046</v>
+        <v>9.26712989985073E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="27">
@@ -776,13 +775,13 @@
         </is>
       </c>
       <c r="B27" s="0">
-        <v>67723496.549</v>
+        <v>67781239.54</v>
       </c>
       <c r="C27" s="0">
-        <v>1549.16020056221</v>
+        <v>1558.3100988115</v>
       </c>
       <c r="D27" s="0">
-        <v>4.57495634308057E-02</v>
+        <v>0.045980572482505</v>
       </c>
     </row>
     <row outlineLevel="0" r="28">
@@ -792,13 +791,13 @@
         </is>
       </c>
       <c r="B28" s="0">
-        <v>24947923.138</v>
+        <v>27088739.999</v>
       </c>
       <c r="C28" s="0">
-        <v>1268.5144436345</v>
+        <v>1362.48512678931</v>
       </c>
       <c r="D28" s="0">
-        <v>0.101692989562111</v>
+        <v>0.100594204591251</v>
       </c>
     </row>
     <row outlineLevel="0" r="29">
@@ -808,13 +807,13 @@
         </is>
       </c>
       <c r="B29" s="0">
-        <v>129730297.061</v>
+        <v>134252770.682</v>
       </c>
       <c r="C29" s="0">
-        <v>3528.13502631276</v>
+        <v>2957.41394610958</v>
       </c>
       <c r="D29" s="0">
-        <v>0.054391843790411</v>
+        <v>4.40573990553194E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="30">
@@ -824,13 +823,13 @@
         </is>
       </c>
       <c r="B30" s="0">
-        <v>43032366.995</v>
+        <v>44400926.002</v>
       </c>
       <c r="C30" s="0">
-        <v>2580.4022936183</v>
+        <v>2465.19217585926</v>
       </c>
       <c r="D30" s="0">
-        <v>0.11992843869909</v>
+        <v>0.111042376717468</v>
       </c>
     </row>
     <row outlineLevel="0" r="31">
@@ -840,13 +839,13 @@
         </is>
       </c>
       <c r="B31" s="0">
-        <v>37910897.991</v>
+        <v>40692718.002</v>
       </c>
       <c r="C31" s="0">
-        <v>606.127367642769</v>
+        <v>508.187131409644</v>
       </c>
       <c r="D31" s="0">
-        <v>3.19764183790457E-02</v>
+        <v>2.49768094323248E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="32">
@@ -856,13 +855,13 @@
         </is>
       </c>
       <c r="B32" s="0">
-        <v>17193229.589</v>
+        <v>18764370.187</v>
       </c>
       <c r="C32" s="0">
-        <v>165.952397125291</v>
+        <v>249.846984031872</v>
       </c>
       <c r="D32" s="0">
-        <v>1.93043891220374E-02</v>
+        <v>2.66299355152315E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="33">
@@ -872,13 +871,13 @@
         </is>
       </c>
       <c r="B33" s="0">
-        <v>61421799.863</v>
+        <v>65039128.884</v>
       </c>
       <c r="C33" s="0">
-        <v>868.469894414692</v>
+        <v>925.399358257796</v>
       </c>
       <c r="D33" s="0">
-        <v>2.82788813206971E-02</v>
+        <v>2.84566959655405E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="34">
@@ -888,13 +887,13 @@
         </is>
       </c>
       <c r="B34" s="0">
-        <v>35073356.999</v>
+        <v>40853345.001</v>
       </c>
       <c r="C34" s="0">
-        <v>1420.79831247798</v>
+        <v>1342.73806852201</v>
       </c>
       <c r="D34" s="0">
-        <v>8.10186668198594E-02</v>
+        <v>6.57345472440089E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="35">
@@ -904,13 +903,13 @@
         </is>
       </c>
       <c r="B35" s="0">
-        <v>41723320.004</v>
+        <v>41832941.006</v>
       </c>
       <c r="C35" s="0">
-        <v>1225.27210110783</v>
+        <v>1055.65823213683</v>
       </c>
       <c r="D35" s="0">
-        <v>5.87332024867804E-02</v>
+        <v>5.04701896041888E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="36">
@@ -920,13 +919,13 @@
         </is>
       </c>
       <c r="B36" s="0">
-        <v>123769709.506</v>
+        <v>124473610.617</v>
       </c>
       <c r="C36" s="0">
-        <v>2805.06233232183</v>
+        <v>3254.53889193084</v>
       </c>
       <c r="D36" s="0">
-        <v>4.53271215310697E-02</v>
+        <v>0.052292833409403</v>
       </c>
     </row>
     <row outlineLevel="0" r="37">
@@ -936,13 +935,13 @@
         </is>
       </c>
       <c r="B37" s="0">
-        <v>125609191.275</v>
+        <v>135802728.736</v>
       </c>
       <c r="C37" s="0">
-        <v>4756.11199354225</v>
+        <v>4751.17746760147</v>
       </c>
       <c r="D37" s="0">
-        <v>7.57287256651394E-02</v>
+        <v>6.99717525829358E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="38">
@@ -952,13 +951,13 @@
         </is>
       </c>
       <c r="B38" s="0">
-        <v>80754585.812</v>
+        <v>84634922.609</v>
       </c>
       <c r="C38" s="0">
-        <v>1083.88674050522</v>
+        <v>1145.03479518491</v>
       </c>
       <c r="D38" s="0">
-        <v>2.68439675494975E-02</v>
+        <v>2.70582109580176E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="39">
@@ -968,13 +967,13 @@
         </is>
       </c>
       <c r="B39" s="0">
-        <v>61016874.601</v>
+        <v>61254900.841</v>
       </c>
       <c r="C39" s="0">
-        <v>417.699081797471</v>
+        <v>630.422444426274</v>
       </c>
       <c r="D39" s="0">
-        <v>1.36912644093582E-02</v>
+        <v>0.020583575706462</v>
       </c>
     </row>
     <row outlineLevel="0" r="40">
@@ -984,13 +983,13 @@
         </is>
       </c>
       <c r="B40" s="0">
-        <v>241279607.04</v>
+        <v>239261130.761</v>
       </c>
       <c r="C40" s="0">
-        <v>-3481.10229203943</v>
+        <v>4519.98306009705</v>
       </c>
       <c r="D40" s="0">
-        <v>-2.88553378774553E-02</v>
+        <v>3.77828445909344E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="41">
@@ -1000,13 +999,13 @@
         </is>
       </c>
       <c r="B41" s="0">
-        <v>18578947.002</v>
+        <v>17762020.003</v>
       </c>
       <c r="C41" s="0">
-        <v>974.653686326561</v>
+        <v>1177.37020638425</v>
       </c>
       <c r="D41" s="0">
-        <v>0.10492022892596</v>
+        <v>0.132571656397796</v>
       </c>
     </row>
     <row outlineLevel="0" r="42">
@@ -1016,13 +1015,13 @@
         </is>
       </c>
       <c r="B42" s="0">
-        <v>9314561.279</v>
+        <v>7804400.21</v>
       </c>
       <c r="C42" s="0">
-        <v>175.825535041237</v>
+        <v>151.577104965722</v>
       </c>
       <c r="D42" s="0">
-        <v>3.77528323180698E-02</v>
+        <v>3.88440112980116E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="43">
@@ -1032,13 +1031,13 @@
         </is>
       </c>
       <c r="B43" s="0">
-        <v>98113946.629</v>
+        <v>98658089.209</v>
       </c>
       <c r="C43" s="0">
-        <v>2149.02302623553</v>
+        <v>2371.74510450447</v>
       </c>
       <c r="D43" s="0">
-        <v>4.38066778490049E-02</v>
+        <v>4.80800940606118E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="44">
@@ -1048,13 +1047,13 @@
         </is>
       </c>
       <c r="B44" s="0">
-        <v>17322408.875</v>
+        <v>17900462.342</v>
       </c>
       <c r="C44" s="0">
-        <v>48.2873787666476</v>
+        <v>40.4139615804159</v>
       </c>
       <c r="D44" s="0">
-        <v>5.57513439557899E-03</v>
+        <v>4.51540980431465E-03</v>
       </c>
     </row>
     <row outlineLevel="0" r="45">
@@ -1064,13 +1063,13 @@
         </is>
       </c>
       <c r="B45" s="0">
-        <v>79057209.281</v>
+        <v>78032791.39</v>
       </c>
       <c r="C45" s="0">
-        <v>2396.81078058055</v>
+        <v>2212.11150389702</v>
       </c>
       <c r="D45" s="0">
-        <v>0.060634844118045</v>
+        <v>5.66969722469905E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="46">
@@ -1080,13 +1079,13 @@
         </is>
       </c>
       <c r="B46" s="0">
-        <v>480614368.135</v>
+        <v>521881132.673</v>
       </c>
       <c r="C46" s="0">
-        <v>11314.8875628397</v>
+        <v>12247.6224126534</v>
       </c>
       <c r="D46" s="0">
-        <v>4.70850990441529E-02</v>
+        <v>4.69364445115035E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="47">
@@ -1096,13 +1095,13 @@
         </is>
       </c>
       <c r="B47" s="0">
-        <v>42560373.008</v>
+        <v>39386042.997</v>
       </c>
       <c r="C47" s="0">
-        <v>1980.51456874864</v>
+        <v>1805.68807574896</v>
       </c>
       <c r="D47" s="0">
-        <v>9.30684779654712E-02</v>
+        <v>9.16917739558906E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="48">
@@ -1112,13 +1111,13 @@
         </is>
       </c>
       <c r="B48" s="0">
-        <v>93103269.048</v>
+        <v>89477324.859</v>
       </c>
       <c r="C48" s="0">
-        <v>1742.6143236367</v>
+        <v>1830.10547298107</v>
       </c>
       <c r="D48" s="0">
-        <v>3.74340093845316E-02</v>
+        <v>4.09065755120638E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="49">
@@ -1128,13 +1127,13 @@
         </is>
       </c>
       <c r="B49" s="0">
-        <v>2107702.867</v>
+        <v>2182637.111</v>
       </c>
       <c r="C49" s="0">
-        <v>50.2888890330636</v>
+        <v>50.8148904793682</v>
       </c>
       <c r="D49" s="0">
-        <v>4.77191446863118E-02</v>
+        <v>4.65628392583197E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="50">
@@ -1144,877 +1143,13 @@
         </is>
       </c>
       <c r="B50" s="0">
-        <v>110808400.626</v>
+        <v>116650629.994</v>
       </c>
       <c r="C50" s="0">
-        <v>744.950612133873</v>
+        <v>1103.72064791259</v>
       </c>
       <c r="D50" s="0">
-        <v>1.34457425235877E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="51">
-      <c r="A51" s="0" t="inlineStr">
-        <is>
-          <t>WI</t>
-        </is>
-      </c>
-      <c r="B51" s="0">
-        <v>64242541.956</v>
-      </c>
-      <c r="C51" s="0">
-        <v>1112.07324669637</v>
-      </c>
-      <c r="D51" s="0">
-        <v>3.46210848088182E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="52">
-      <c r="A52" s="0" t="inlineStr">
-        <is>
-          <t>WV</t>
-        </is>
-      </c>
-      <c r="B52" s="0">
-        <v>65836062.988</v>
-      </c>
-      <c r="C52" s="0">
-        <v>5418.00410780477</v>
-      </c>
-      <c r="D52" s="0">
-        <v>0.164590768703539</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="53">
-      <c r="A53" s="0" t="inlineStr">
-        <is>
-          <t>WY</t>
-        </is>
-      </c>
-      <c r="B53" s="0">
-        <v>43460743.876</v>
-      </c>
-      <c r="C53" s="0">
-        <v>1758.57047677893</v>
-      </c>
-      <c r="D53" s="0">
-        <v>8.09268466180145E-02</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D53"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row outlineLevel="0" r="1">
-      <c r="A1" s="0" t="inlineStr">
-        <is>
-          <t>PSTATABB</t>
-        </is>
-      </c>
-      <c r="B1" s="0" t="inlineStr">
-        <is>
-          <t>SumOfPLNGENAN</t>
-        </is>
-      </c>
-      <c r="C1" s="0" t="inlineStr">
-        <is>
-          <t>SumOfPLPM25AN2</t>
-        </is>
-      </c>
-      <c r="D1" s="0" t="inlineStr">
-        <is>
-          <t>STPM25RTA</t>
-        </is>
-      </c>
-    </row>
-    <row outlineLevel="0" r="2">
-      <c r="A2" s="0" t="inlineStr">
-        <is>
-          <t>AK</t>
-        </is>
-      </c>
-      <c r="B2" s="0">
-        <v>6694128.234</v>
-      </c>
-      <c r="C2" s="0">
-        <v>1183.97361602816</v>
-      </c>
-      <c r="D2" s="0">
-        <v>0.353734967314987</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="3">
-      <c r="A3" s="0" t="inlineStr">
-        <is>
-          <t>AL</t>
-        </is>
-      </c>
-      <c r="B3" s="0">
-        <v>144788892.892</v>
-      </c>
-      <c r="C3" s="0">
-        <v>1940.07988943241</v>
-      </c>
-      <c r="D3" s="0">
-        <v>2.67987391944428E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="4">
-      <c r="A4" s="0" t="inlineStr">
-        <is>
-          <t>AR</t>
-        </is>
-      </c>
-      <c r="B4" s="0">
-        <v>65905029.856</v>
-      </c>
-      <c r="C4" s="0">
-        <v>2484.18914916171</v>
-      </c>
-      <c r="D4" s="0">
-        <v>7.53869364626516E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="5">
-      <c r="A5" s="0" t="inlineStr">
-        <is>
-          <t>AZ</t>
-        </is>
-      </c>
-      <c r="B5" s="0">
-        <v>104698773.165</v>
-      </c>
-      <c r="C5" s="0">
-        <v>2033.02842595787</v>
-      </c>
-      <c r="D5" s="0">
-        <v>3.88357640591246E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="6">
-      <c r="A6" s="0" t="inlineStr">
-        <is>
-          <t>CA</t>
-        </is>
-      </c>
-      <c r="B6" s="0">
-        <v>203256382.497</v>
-      </c>
-      <c r="C6" s="0">
-        <v>3498.63642830383</v>
-      </c>
-      <c r="D6" s="0">
-        <v>3.44258456765113E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="7">
-      <c r="A7" s="0" t="inlineStr">
-        <is>
-          <t>CO</t>
-        </is>
-      </c>
-      <c r="B7" s="0">
-        <v>58012255.357</v>
-      </c>
-      <c r="C7" s="0">
-        <v>1270.69109002107</v>
-      </c>
-      <c r="D7" s="0">
-        <v>4.38076776088571E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="8">
-      <c r="A8" s="0" t="inlineStr">
-        <is>
-          <t>CT</t>
-        </is>
-      </c>
-      <c r="B8" s="0">
-        <v>42761369.034</v>
-      </c>
-      <c r="C8" s="0">
-        <v>378.586212088675</v>
-      </c>
-      <c r="D8" s="0">
-        <v>1.77069266321972E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="9">
-      <c r="A9" s="0" t="inlineStr">
-        <is>
-          <t>DC</t>
-        </is>
-      </c>
-      <c r="B9" s="0">
-        <v>160237.001</v>
-      </c>
-      <c r="C9" s="0">
-        <v>7.9055459044218</v>
-      </c>
-      <c r="D9" s="0">
-        <v>9.86731635650345E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="10">
-      <c r="A10" s="0" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="B10" s="0">
-        <v>5308370</v>
-      </c>
-      <c r="C10" s="0">
-        <v>250.879158350828</v>
-      </c>
-      <c r="D10" s="0">
-        <v>9.45221069182547E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="11">
-      <c r="A11" s="0" t="inlineStr">
-        <is>
-          <t>FL</t>
-        </is>
-      </c>
-      <c r="B11" s="0">
-        <v>257955504.155</v>
-      </c>
-      <c r="C11" s="0">
-        <v>8203.02615556563</v>
-      </c>
-      <c r="D11" s="0">
-        <v>6.36003188413193E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="12">
-      <c r="A12" s="0" t="inlineStr">
-        <is>
-          <t>GA</t>
-        </is>
-      </c>
-      <c r="B12" s="0">
-        <v>126484632.485</v>
-      </c>
-      <c r="C12" s="0">
-        <v>2862.14913314853</v>
-      </c>
-      <c r="D12" s="0">
-        <v>4.52568676038641E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="13">
-      <c r="A13" s="0" t="inlineStr">
-        <is>
-          <t>HI</t>
-        </is>
-      </c>
-      <c r="B13" s="0">
-        <v>9304192.004</v>
-      </c>
-      <c r="C13" s="0">
-        <v>2868.72291279245</v>
-      </c>
-      <c r="D13" s="0">
-        <v>0.61665170098793</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="14">
-      <c r="A14" s="0" t="inlineStr">
-        <is>
-          <t>IA</t>
-        </is>
-      </c>
-      <c r="B14" s="0">
-        <v>72909386.062</v>
-      </c>
-      <c r="C14" s="0">
-        <v>1322.48062588143</v>
-      </c>
-      <c r="D14" s="0">
-        <v>3.62773765439975E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="15">
-      <c r="A15" s="0" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B15" s="0">
-        <v>16278410.189</v>
-      </c>
-      <c r="C15" s="0">
-        <v>149.872489678535</v>
-      </c>
-      <c r="D15" s="0">
-        <v>1.84136519400168E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="16">
-      <c r="A16" s="0" t="inlineStr">
-        <is>
-          <t>IL</t>
-        </is>
-      </c>
-      <c r="B16" s="0">
-        <v>185197549.577</v>
-      </c>
-      <c r="C16" s="0">
-        <v>1949.41923545194</v>
-      </c>
-      <c r="D16" s="0">
-        <v>2.10523221274202E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="17">
-      <c r="A17" s="0" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="B17" s="0">
-        <v>98022168.549</v>
-      </c>
-      <c r="C17" s="0">
-        <v>5230.59915954845</v>
-      </c>
-      <c r="D17" s="0">
-        <v>0.106722779897156</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="18">
-      <c r="A18" s="0" t="inlineStr">
-        <is>
-          <t>KS</t>
-        </is>
-      </c>
-      <c r="B18" s="0">
-        <v>62194840.58</v>
-      </c>
-      <c r="C18" s="0">
-        <v>1064.90544996322</v>
-      </c>
-      <c r="D18" s="0">
-        <v>3.42441733118827E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="19">
-      <c r="A19" s="0" t="inlineStr">
-        <is>
-          <t>KY</t>
-        </is>
-      </c>
-      <c r="B19" s="0">
-        <v>69146933.093</v>
-      </c>
-      <c r="C19" s="0">
-        <v>3194.50009645734</v>
-      </c>
-      <c r="D19" s="0">
-        <v>9.23974485509244E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="20">
-      <c r="A20" s="0" t="inlineStr">
-        <is>
-          <t>LA</t>
-        </is>
-      </c>
-      <c r="B20" s="0">
-        <v>105223371.518</v>
-      </c>
-      <c r="C20" s="0">
-        <v>3016.95527741294</v>
-      </c>
-      <c r="D20" s="0">
-        <v>5.73438245494129E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="21">
-      <c r="A21" s="0" t="inlineStr">
-        <is>
-          <t>MA</t>
-        </is>
-      </c>
-      <c r="B21" s="0">
-        <v>21022930.789</v>
-      </c>
-      <c r="C21" s="0">
-        <v>1178.77096474409</v>
-      </c>
-      <c r="D21" s="0">
-        <v>0.112141449408268</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="22">
-      <c r="A22" s="0" t="inlineStr">
-        <is>
-          <t>MD</t>
-        </is>
-      </c>
-      <c r="B22" s="0">
-        <v>37134094.879</v>
-      </c>
-      <c r="C22" s="0">
-        <v>422.192780720041</v>
-      </c>
-      <c r="D22" s="0">
-        <v>2.27388216729526E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="23">
-      <c r="A23" s="0" t="inlineStr">
-        <is>
-          <t>ME</t>
-        </is>
-      </c>
-      <c r="B23" s="0">
-        <v>12763920.003</v>
-      </c>
-      <c r="C23" s="0">
-        <v>692.629064792758</v>
-      </c>
-      <c r="D23" s="0">
-        <v>0.108529208053633</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="24">
-      <c r="A24" s="0" t="inlineStr">
-        <is>
-          <t>MI</t>
-        </is>
-      </c>
-      <c r="B24" s="0">
-        <v>116615130.596</v>
-      </c>
-      <c r="C24" s="0">
-        <v>3355.50434569066</v>
-      </c>
-      <c r="D24" s="0">
-        <v>5.75483529202642E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="25">
-      <c r="A25" s="0" t="inlineStr">
-        <is>
-          <t>MN</t>
-        </is>
-      </c>
-      <c r="B25" s="0">
-        <v>58966891.046</v>
-      </c>
-      <c r="C25" s="0">
-        <v>1046.45288600298</v>
-      </c>
-      <c r="D25" s="0">
-        <v>3.54928966896574E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="26">
-      <c r="A26" s="0" t="inlineStr">
-        <is>
-          <t>MO</t>
-        </is>
-      </c>
-      <c r="B26" s="0">
-        <v>79361031.625</v>
-      </c>
-      <c r="C26" s="0">
-        <v>3677.24494527519</v>
-      </c>
-      <c r="D26" s="0">
-        <v>9.26712989985073E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="27">
-      <c r="A27" s="0" t="inlineStr">
-        <is>
-          <t>MS</t>
-        </is>
-      </c>
-      <c r="B27" s="0">
-        <v>67781239.54</v>
-      </c>
-      <c r="C27" s="0">
-        <v>1558.3100988115</v>
-      </c>
-      <c r="D27" s="0">
-        <v>0.045980572482505</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="28">
-      <c r="A28" s="0" t="inlineStr">
-        <is>
-          <t>MT</t>
-        </is>
-      </c>
-      <c r="B28" s="0">
-        <v>27088739.999</v>
-      </c>
-      <c r="C28" s="0">
-        <v>1362.48518488605</v>
-      </c>
-      <c r="D28" s="0">
-        <v>0.100594208880616</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="29">
-      <c r="A29" s="0" t="inlineStr">
-        <is>
-          <t>NC</t>
-        </is>
-      </c>
-      <c r="B29" s="0">
-        <v>134252770.682</v>
-      </c>
-      <c r="C29" s="0">
-        <v>2957.41394610958</v>
-      </c>
-      <c r="D29" s="0">
-        <v>4.40573990553194E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="30">
-      <c r="A30" s="0" t="inlineStr">
-        <is>
-          <t>ND</t>
-        </is>
-      </c>
-      <c r="B30" s="0">
-        <v>44400926.002</v>
-      </c>
-      <c r="C30" s="0">
-        <v>2465.19217585926</v>
-      </c>
-      <c r="D30" s="0">
-        <v>0.111042376717468</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="31">
-      <c r="A31" s="0" t="inlineStr">
-        <is>
-          <t>NE</t>
-        </is>
-      </c>
-      <c r="B31" s="0">
-        <v>40692718.002</v>
-      </c>
-      <c r="C31" s="0">
-        <v>508.187131409644</v>
-      </c>
-      <c r="D31" s="0">
-        <v>2.49768094323248E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="32">
-      <c r="A32" s="0" t="inlineStr">
-        <is>
-          <t>NH</t>
-        </is>
-      </c>
-      <c r="B32" s="0">
-        <v>18764370.187</v>
-      </c>
-      <c r="C32" s="0">
-        <v>249.985244907066</v>
-      </c>
-      <c r="D32" s="0">
-        <v>2.66446720476934E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="33">
-      <c r="A33" s="0" t="inlineStr">
-        <is>
-          <t>NJ</t>
-        </is>
-      </c>
-      <c r="B33" s="0">
-        <v>65039128.884</v>
-      </c>
-      <c r="C33" s="0">
-        <v>933.43284055604</v>
-      </c>
-      <c r="D33" s="0">
-        <v>2.87037313252106E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="34">
-      <c r="A34" s="0" t="inlineStr">
-        <is>
-          <t>NM</t>
-        </is>
-      </c>
-      <c r="B34" s="0">
-        <v>40853345.001</v>
-      </c>
-      <c r="C34" s="0">
-        <v>1342.73806852201</v>
-      </c>
-      <c r="D34" s="0">
-        <v>6.57345472440089E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="35">
-      <c r="A35" s="0" t="inlineStr">
-        <is>
-          <t>NV</t>
-        </is>
-      </c>
-      <c r="B35" s="0">
-        <v>41832941.006</v>
-      </c>
-      <c r="C35" s="0">
-        <v>1055.65823213683</v>
-      </c>
-      <c r="D35" s="0">
-        <v>5.04701896041888E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="36">
-      <c r="A36" s="0" t="inlineStr">
-        <is>
-          <t>NY</t>
-        </is>
-      </c>
-      <c r="B36" s="0">
-        <v>124473610.617</v>
-      </c>
-      <c r="C36" s="0">
-        <v>3302.5195336783</v>
-      </c>
-      <c r="D36" s="0">
-        <v>5.30637701808138E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="37">
-      <c r="A37" s="0" t="inlineStr">
-        <is>
-          <t>OH</t>
-        </is>
-      </c>
-      <c r="B37" s="0">
-        <v>135802728.736</v>
-      </c>
-      <c r="C37" s="0">
-        <v>4751.17751565147</v>
-      </c>
-      <c r="D37" s="0">
-        <v>6.99717532905799E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="38">
-      <c r="A38" s="0" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="B38" s="0">
-        <v>84634922.609</v>
-      </c>
-      <c r="C38" s="0">
-        <v>1145.03479518491</v>
-      </c>
-      <c r="D38" s="0">
-        <v>2.70582109580176E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="39">
-      <c r="A39" s="0" t="inlineStr">
-        <is>
-          <t>OR</t>
-        </is>
-      </c>
-      <c r="B39" s="0">
-        <v>61254900.841</v>
-      </c>
-      <c r="C39" s="0">
-        <v>650.200533395698</v>
-      </c>
-      <c r="D39" s="0">
-        <v>2.12293391865389E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="40">
-      <c r="A40" s="0" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
-      <c r="B40" s="0">
-        <v>239261130.761</v>
-      </c>
-      <c r="C40" s="0">
-        <v>-3260.37040673113</v>
-      </c>
-      <c r="D40" s="0">
-        <v>-2.72536570930775E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="41">
-      <c r="A41" s="0" t="inlineStr">
-        <is>
-          <t>PR</t>
-        </is>
-      </c>
-      <c r="B41" s="0">
-        <v>17762020.003</v>
-      </c>
-      <c r="C41" s="0">
-        <v>1177.37020638425</v>
-      </c>
-      <c r="D41" s="0">
-        <v>0.132571656397796</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="42">
-      <c r="A42" s="0" t="inlineStr">
-        <is>
-          <t>RI</t>
-        </is>
-      </c>
-      <c r="B42" s="0">
-        <v>7804400.21</v>
-      </c>
-      <c r="C42" s="0">
-        <v>151.577104965722</v>
-      </c>
-      <c r="D42" s="0">
-        <v>3.88440112980116E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="43">
-      <c r="A43" s="0" t="inlineStr">
-        <is>
-          <t>SC</t>
-        </is>
-      </c>
-      <c r="B43" s="0">
-        <v>98658089.209</v>
-      </c>
-      <c r="C43" s="0">
-        <v>2371.74510450447</v>
-      </c>
-      <c r="D43" s="0">
-        <v>4.80800940606118E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="44">
-      <c r="A44" s="0" t="inlineStr">
-        <is>
-          <t>SD</t>
-        </is>
-      </c>
-      <c r="B44" s="0">
-        <v>17900462.342</v>
-      </c>
-      <c r="C44" s="0">
-        <v>40.4139615804159</v>
-      </c>
-      <c r="D44" s="0">
-        <v>4.51540980431465E-03</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="45">
-      <c r="A45" s="0" t="inlineStr">
-        <is>
-          <t>TN</t>
-        </is>
-      </c>
-      <c r="B45" s="0">
-        <v>78032791.39</v>
-      </c>
-      <c r="C45" s="0">
-        <v>2212.11150389702</v>
-      </c>
-      <c r="D45" s="0">
-        <v>5.66969722469905E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="46">
-      <c r="A46" s="0" t="inlineStr">
-        <is>
-          <t>TX</t>
-        </is>
-      </c>
-      <c r="B46" s="0">
-        <v>521881132.673</v>
-      </c>
-      <c r="C46" s="0">
-        <v>12250.8913675252</v>
-      </c>
-      <c r="D46" s="0">
-        <v>4.69489720955342E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="47">
-      <c r="A47" s="0" t="inlineStr">
-        <is>
-          <t>UT</t>
-        </is>
-      </c>
-      <c r="B47" s="0">
-        <v>39386042.997</v>
-      </c>
-      <c r="C47" s="0">
-        <v>1805.68807574896</v>
-      </c>
-      <c r="D47" s="0">
-        <v>9.16917739558906E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="48">
-      <c r="A48" s="0" t="inlineStr">
-        <is>
-          <t>VA</t>
-        </is>
-      </c>
-      <c r="B48" s="0">
-        <v>89477324.859</v>
-      </c>
-      <c r="C48" s="0">
-        <v>1864.4399108766</v>
-      </c>
-      <c r="D48" s="0">
-        <v>4.16740199556618E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="49">
-      <c r="A49" s="0" t="inlineStr">
-        <is>
-          <t>VT</t>
-        </is>
-      </c>
-      <c r="B49" s="0">
-        <v>2182637.111</v>
-      </c>
-      <c r="C49" s="0">
-        <v>50.8148904793682</v>
-      </c>
-      <c r="D49" s="0">
-        <v>4.65628392583197E-02</v>
-      </c>
-    </row>
-    <row outlineLevel="0" r="50">
-      <c r="A50" s="0" t="inlineStr">
-        <is>
-          <t>WA</t>
-        </is>
-      </c>
-      <c r="B50" s="0">
-        <v>116650629.994</v>
-      </c>
-      <c r="C50" s="0">
-        <v>1103.75548087203</v>
-      </c>
-      <c r="D50" s="0">
-        <v>1.89241237861948E-02</v>
+        <v>1.89235265676553E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="51">
@@ -2342,22 +1477,29 @@
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
-    <TaxCatchAll xmlns="6c854b04-c9c6-4391-adbe-2e73191270e7" xsi:nil="true"/>
+    <SharedWithUsers xmlns="c05e7bd6-26a7-41a1-805c-893279a3732f">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="059b9c67-646b-4b4e-9ab1-2b1c805d0390">
       <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="6c854b04-c9c6-4391-adbe-2e73191270e7" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{96B8852E-CB39-48CB-9156-BDBD868199A4}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{975E3D7B-67F5-43EA-A2E4-930EC9CAF4A5}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{08BCE0E9-C5FC-43DC-BFE9-B81CCC382F29}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CBBD9D4-15C2-4F45-B37E-132DA4C3F68B}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4C9718D7-70E0-4149-BB06-99C9C0FA79DF}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D4E802E0-D20C-4067-949A-6D485BDB8B14}"/>
 </file>
</xml_diff>

<commit_message>
Updating Access 2022 QA Data
</commit_message>
<xml_diff>
--- a/data/2b_pm_nh3_voc/static_tables/qa/2022/eGRID2022_pmemissions_state.xlsx
+++ b/data/2b_pm_nh3_voc/static_tables/qa/2022/eGRID2022_pmemissions_state.xlsx
@@ -378,10 +378,10 @@
         <v>6694128.234</v>
       </c>
       <c r="C2" s="0">
-        <v>1183.97349245646</v>
+        <v>1183.97361602816</v>
       </c>
       <c r="D2" s="0">
-        <v>0.353734930395556</v>
+        <v>0.353734967314986</v>
       </c>
     </row>
     <row outlineLevel="0" r="3">
@@ -442,10 +442,10 @@
         <v>203256382.497</v>
       </c>
       <c r="C6" s="0">
-        <v>3495.27080754069</v>
+        <v>3498.63642830383</v>
       </c>
       <c r="D6" s="0">
-        <v>3.43927286769682E-02</v>
+        <v>3.44258456765113E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="7">
@@ -474,10 +474,10 @@
         <v>42761369.034</v>
       </c>
       <c r="C8" s="0">
-        <v>331.922671179937</v>
+        <v>369.872453021623</v>
       </c>
       <c r="D8" s="0">
-        <v>1.55244174205939E-02</v>
+        <v>1.72993737748449E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="9">
@@ -522,10 +522,10 @@
         <v>257955504.155</v>
       </c>
       <c r="C11" s="0">
-        <v>8169.759739289</v>
+        <v>8421.89142857893</v>
       </c>
       <c r="D11" s="0">
-        <v>6.33423951626941E-02</v>
+        <v>6.52972415236264E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="12">
@@ -554,10 +554,10 @@
         <v>9304192.004</v>
       </c>
       <c r="C13" s="0">
-        <v>2863.11047610233</v>
+        <v>2868.72291279245</v>
       </c>
       <c r="D13" s="0">
-        <v>0.615445269158555</v>
+        <v>0.61665170098793</v>
       </c>
     </row>
     <row outlineLevel="0" r="14">
@@ -570,10 +570,10 @@
         <v>72909386.062</v>
       </c>
       <c r="C14" s="0">
-        <v>1322.48058061623</v>
+        <v>1322.48062588143</v>
       </c>
       <c r="D14" s="0">
-        <v>3.62773753023139E-02</v>
+        <v>3.62773765439975E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="15">
@@ -666,10 +666,10 @@
         <v>105223371.518</v>
       </c>
       <c r="C20" s="0">
-        <v>3010.29752047694</v>
+        <v>3016.95527741294</v>
       </c>
       <c r="D20" s="0">
-        <v>5.72172793372618E-02</v>
+        <v>5.73438245494129E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="21">
@@ -682,10 +682,10 @@
         <v>21022930.789</v>
       </c>
       <c r="C21" s="0">
-        <v>1106.48090345667</v>
+        <v>1183.82944330613</v>
       </c>
       <c r="D21" s="0">
-        <v>0.105264191235945</v>
+        <v>0.112622683791126</v>
       </c>
     </row>
     <row outlineLevel="0" r="22">
@@ -698,10 +698,10 @@
         <v>37134094.879</v>
       </c>
       <c r="C22" s="0">
-        <v>408.052402065771</v>
+        <v>419.435827220912</v>
       </c>
       <c r="D22" s="0">
-        <v>2.19772370052586E-02</v>
+        <v>0.022590335301702</v>
       </c>
     </row>
     <row outlineLevel="0" r="23">
@@ -714,10 +714,10 @@
         <v>12763920.003</v>
       </c>
       <c r="C23" s="0">
-        <v>691.622991673066</v>
+        <v>692.629064792758</v>
       </c>
       <c r="D23" s="0">
-        <v>0.108371564771717</v>
+        <v>0.108529208053633</v>
       </c>
     </row>
     <row outlineLevel="0" r="24">
@@ -730,10 +730,10 @@
         <v>116615130.596</v>
       </c>
       <c r="C24" s="0">
-        <v>3355.34714861007</v>
+        <v>3355.59493001565</v>
       </c>
       <c r="D24" s="0">
-        <v>5.75456569222444E-02</v>
+        <v>5.75499064806734E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="25">
@@ -746,10 +746,10 @@
         <v>58966891.046</v>
       </c>
       <c r="C25" s="0">
-        <v>1041.80325738326</v>
+        <v>1046.45288600298</v>
       </c>
       <c r="D25" s="0">
-        <v>3.53351936621706E-02</v>
+        <v>3.54928966896574E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="26">
@@ -794,10 +794,10 @@
         <v>27088739.999</v>
       </c>
       <c r="C28" s="0">
-        <v>1362.48512678931</v>
+        <v>1362.48803162631</v>
       </c>
       <c r="D28" s="0">
-        <v>0.100594204591251</v>
+        <v>0.100594419059477</v>
       </c>
     </row>
     <row outlineLevel="0" r="29">
@@ -858,10 +858,10 @@
         <v>18764370.187</v>
       </c>
       <c r="C32" s="0">
-        <v>249.846984031872</v>
+        <v>249.985244907066</v>
       </c>
       <c r="D32" s="0">
-        <v>2.66299355152315E-02</v>
+        <v>2.66446720476934E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="33">
@@ -874,10 +874,10 @@
         <v>65039128.884</v>
       </c>
       <c r="C33" s="0">
-        <v>925.399358257796</v>
+        <v>933.43284055604</v>
       </c>
       <c r="D33" s="0">
-        <v>2.84566959655405E-02</v>
+        <v>2.87037313252106E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="34">
@@ -922,10 +922,10 @@
         <v>124473610.617</v>
       </c>
       <c r="C36" s="0">
-        <v>3254.53889193084</v>
+        <v>3289.61545460296</v>
       </c>
       <c r="D36" s="0">
-        <v>0.052292833409403</v>
+        <v>5.28564317897866E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="37">
@@ -938,10 +938,10 @@
         <v>135802728.736</v>
       </c>
       <c r="C37" s="0">
-        <v>4751.17746760147</v>
+        <v>4751.17751565147</v>
       </c>
       <c r="D37" s="0">
-        <v>6.99717525829358E-02</v>
+        <v>6.99717532905799E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="38">
@@ -970,10 +970,10 @@
         <v>61254900.841</v>
       </c>
       <c r="C39" s="0">
-        <v>630.422444426274</v>
+        <v>742.603908797989</v>
       </c>
       <c r="D39" s="0">
-        <v>0.020583575706462</v>
+        <v>2.42463508585403E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="40">
@@ -986,10 +986,10 @@
         <v>239261130.761</v>
       </c>
       <c r="C40" s="0">
-        <v>4519.98306009705</v>
+        <v>4535.00448365747</v>
       </c>
       <c r="D40" s="0">
-        <v>3.77828445909344E-02</v>
+        <v>3.79084096880535E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="41">
@@ -1082,10 +1082,10 @@
         <v>521881132.673</v>
       </c>
       <c r="C46" s="0">
-        <v>12247.6224126534</v>
+        <v>12250.8913675252</v>
       </c>
       <c r="D46" s="0">
-        <v>4.69364445115035E-02</v>
+        <v>4.69489720955342E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="47">
@@ -1114,10 +1114,10 @@
         <v>89477324.859</v>
       </c>
       <c r="C48" s="0">
-        <v>1830.10547298107</v>
+        <v>1865.5709765427</v>
       </c>
       <c r="D48" s="0">
-        <v>4.09065755120638E-02</v>
+        <v>4.16993015712641E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="49">
@@ -1146,10 +1146,10 @@
         <v>116650629.994</v>
       </c>
       <c r="C50" s="0">
-        <v>1103.72064791259</v>
+        <v>1103.75548087203</v>
       </c>
       <c r="D50" s="0">
-        <v>1.89235265676553E-02</v>
+        <v>1.89241237861948E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="51">
@@ -1477,29 +1477,22 @@
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
-    <SharedWithUsers xmlns="c05e7bd6-26a7-41a1-805c-893279a3732f">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
+    <TaxCatchAll xmlns="6c854b04-c9c6-4391-adbe-2e73191270e7" xsi:nil="true"/>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="059b9c67-646b-4b4e-9ab1-2b1c805d0390">
       <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="6c854b04-c9c6-4391-adbe-2e73191270e7" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{975E3D7B-67F5-43EA-A2E4-930EC9CAF4A5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38083C74-77D1-44FA-B8A8-419E942AEE5F}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CBBD9D4-15C2-4F45-B37E-132DA4C3F68B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1104ACA0-50ED-4B60-ACE5-F0C67785AE73}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D4E802E0-D20C-4067-949A-6D485BDB8B14}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DD397F47-8914-4322-B35C-BAF7E9ADE317}"/>
 </file>
</xml_diff>

<commit_message>
Updating QA static tables for 2021 and 2022
</commit_message>
<xml_diff>
--- a/data/2b_pm_nh3_voc/static_tables/qa/2022/eGRID2022_pmemissions_state.xlsx
+++ b/data/2b_pm_nh3_voc/static_tables/qa/2022/eGRID2022_pmemissions_state.xlsx
@@ -378,10 +378,10 @@
         <v>6694128.234</v>
       </c>
       <c r="C2" s="0">
-        <v>1183.97361602816</v>
+        <v>1183.94290293087</v>
       </c>
       <c r="D2" s="0">
-        <v>0.353734967314986</v>
+        <v>0.35372579118444</v>
       </c>
     </row>
     <row outlineLevel="0" r="3">
@@ -394,10 +394,10 @@
         <v>144788892.892</v>
       </c>
       <c r="C3" s="0">
-        <v>1940.07988943241</v>
+        <v>1940.03229978583</v>
       </c>
       <c r="D3" s="0">
-        <v>2.67987391944428E-02</v>
+        <v>0.026798081828458</v>
       </c>
     </row>
     <row outlineLevel="0" r="4">
@@ -410,10 +410,10 @@
         <v>65905029.856</v>
       </c>
       <c r="C4" s="0">
-        <v>2484.18914916171</v>
+        <v>2484.18112495628</v>
       </c>
       <c r="D4" s="0">
-        <v>7.53869364626516E-02</v>
+        <v>7.53866929545173E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="5">
@@ -426,10 +426,10 @@
         <v>104698773.165</v>
       </c>
       <c r="C5" s="0">
-        <v>2033.02842595787</v>
+        <v>2032.93956367084</v>
       </c>
       <c r="D5" s="0">
-        <v>3.88357640591246E-02</v>
+        <v>3.88340665743433E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="6">
@@ -442,10 +442,10 @@
         <v>203256382.497</v>
       </c>
       <c r="C6" s="0">
-        <v>3498.63642830383</v>
+        <v>3498.03531080828</v>
       </c>
       <c r="D6" s="0">
-        <v>3.44258456765113E-02</v>
+        <v>3.44199308069444E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="7">
@@ -458,10 +458,10 @@
         <v>58012255.357</v>
       </c>
       <c r="C7" s="0">
-        <v>1270.69109002107</v>
+        <v>1270.67934253213</v>
       </c>
       <c r="D7" s="0">
-        <v>4.38076776088571E-02</v>
+        <v>4.38072726086075E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="8">
@@ -474,10 +474,10 @@
         <v>42761369.034</v>
       </c>
       <c r="C8" s="0">
-        <v>369.872453021623</v>
+        <v>369.838410006589</v>
       </c>
       <c r="D8" s="0">
-        <v>1.72993737748449E-02</v>
+        <v>1.72977815426127E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="9">
@@ -490,10 +490,10 @@
         <v>160237.001</v>
       </c>
       <c r="C9" s="0">
-        <v>7.9055459044218</v>
+        <v>7.8967833554366</v>
       </c>
       <c r="D9" s="0">
-        <v>9.86731635650345E-02</v>
+        <v>9.85637937075045E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="10">
@@ -522,10 +522,10 @@
         <v>257955504.155</v>
       </c>
       <c r="C11" s="0">
-        <v>8421.89142857893</v>
+        <v>8421.76355201544</v>
       </c>
       <c r="D11" s="0">
-        <v>6.52972415236264E-02</v>
+        <v>6.52962500614446E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="12">
@@ -538,10 +538,10 @@
         <v>126484632.485</v>
       </c>
       <c r="C12" s="0">
-        <v>2862.14913314853</v>
+        <v>2862.12487116497</v>
       </c>
       <c r="D12" s="0">
-        <v>4.52568676038641E-02</v>
+        <v>4.52564839685863E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="13">
@@ -570,10 +570,10 @@
         <v>72909386.062</v>
       </c>
       <c r="C14" s="0">
-        <v>1322.48062588143</v>
+        <v>1322.47055757701</v>
       </c>
       <c r="D14" s="0">
-        <v>3.62773765439975E-02</v>
+        <v>3.62771003572137E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="15">
@@ -586,10 +586,10 @@
         <v>16278410.189</v>
       </c>
       <c r="C15" s="0">
-        <v>149.872489678535</v>
+        <v>149.87017233589</v>
       </c>
       <c r="D15" s="0">
-        <v>1.84136519400168E-02</v>
+        <v>1.84133672263847E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="16">
@@ -602,10 +602,10 @@
         <v>185197549.577</v>
       </c>
       <c r="C16" s="0">
-        <v>1949.41923545194</v>
+        <v>1949.38579780069</v>
       </c>
       <c r="D16" s="0">
-        <v>2.10523221274202E-02</v>
+        <v>2.10519610248967E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="17">
@@ -618,10 +618,10 @@
         <v>98022168.549</v>
       </c>
       <c r="C17" s="0">
-        <v>5230.59915954845</v>
+        <v>5230.45865838915</v>
       </c>
       <c r="D17" s="0">
-        <v>0.106722779897156</v>
+        <v>0.106719913175039</v>
       </c>
     </row>
     <row outlineLevel="0" r="18">
@@ -634,10 +634,10 @@
         <v>62194840.58</v>
       </c>
       <c r="C18" s="0">
-        <v>1064.90544996322</v>
+        <v>1064.88016313854</v>
       </c>
       <c r="D18" s="0">
-        <v>3.42441733118827E-02</v>
+        <v>3.42433601632535E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="19">
@@ -650,10 +650,10 @@
         <v>69146933.093</v>
       </c>
       <c r="C19" s="0">
-        <v>3194.50009645734</v>
+        <v>3194.5000915954</v>
       </c>
       <c r="D19" s="0">
-        <v>9.23974485509244E-02</v>
+        <v>9.23974484102981E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="20">
@@ -666,10 +666,10 @@
         <v>105223371.518</v>
       </c>
       <c r="C20" s="0">
-        <v>3016.95527741294</v>
+        <v>3016.54525313579</v>
       </c>
       <c r="D20" s="0">
-        <v>5.73438245494129E-02</v>
+        <v>5.73360311424685E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="21">
@@ -682,10 +682,10 @@
         <v>21022930.789</v>
       </c>
       <c r="C21" s="0">
-        <v>1183.82944330613</v>
+        <v>1183.79236409571</v>
       </c>
       <c r="D21" s="0">
-        <v>0.112622683791126</v>
+        <v>0.11261915628958</v>
       </c>
     </row>
     <row outlineLevel="0" r="22">
@@ -698,10 +698,10 @@
         <v>37134094.879</v>
       </c>
       <c r="C22" s="0">
-        <v>419.435827220912</v>
+        <v>406.793956145626</v>
       </c>
       <c r="D22" s="0">
-        <v>0.022590335301702</v>
+        <v>2.19094585432147E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="23">
@@ -714,10 +714,10 @@
         <v>12763920.003</v>
       </c>
       <c r="C23" s="0">
-        <v>692.629064792758</v>
+        <v>692.627123939482</v>
       </c>
       <c r="D23" s="0">
-        <v>0.108529208053633</v>
+        <v>0.108528903938083</v>
       </c>
     </row>
     <row outlineLevel="0" r="24">
@@ -730,10 +730,10 @@
         <v>116615130.596</v>
       </c>
       <c r="C24" s="0">
-        <v>3355.59493001565</v>
+        <v>3355.55815259612</v>
       </c>
       <c r="D24" s="0">
-        <v>5.75499064806734E-02</v>
+        <v>5.75492757319986E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="25">
@@ -746,10 +746,10 @@
         <v>58966891.046</v>
       </c>
       <c r="C25" s="0">
-        <v>1046.45288600298</v>
+        <v>1046.4296742071</v>
       </c>
       <c r="D25" s="0">
-        <v>3.54928966896574E-02</v>
+        <v>3.54921094073209E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="26">
@@ -762,10 +762,10 @@
         <v>79361031.625</v>
       </c>
       <c r="C26" s="0">
-        <v>3677.24494527519</v>
+        <v>3677.22079286612</v>
       </c>
       <c r="D26" s="0">
-        <v>9.26712989985073E-02</v>
+        <v>9.26706903267556E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="27">
@@ -778,10 +778,10 @@
         <v>67781239.54</v>
       </c>
       <c r="C27" s="0">
-        <v>1558.3100988115</v>
+        <v>1558.28745952162</v>
       </c>
       <c r="D27" s="0">
-        <v>0.045980572482505</v>
+        <v>4.59799044720043E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="28">
@@ -794,10 +794,10 @@
         <v>27088739.999</v>
       </c>
       <c r="C28" s="0">
-        <v>1362.48803162631</v>
+        <v>1362.4879205328</v>
       </c>
       <c r="D28" s="0">
-        <v>0.100594419059477</v>
+        <v>0.100594410857286</v>
       </c>
     </row>
     <row outlineLevel="0" r="29">
@@ -810,10 +810,10 @@
         <v>134252770.682</v>
       </c>
       <c r="C29" s="0">
-        <v>2957.41394610958</v>
+        <v>2957.40014388358</v>
       </c>
       <c r="D29" s="0">
-        <v>4.40573990553194E-02</v>
+        <v>4.40571934398088E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="30">
@@ -826,10 +826,10 @@
         <v>44400926.002</v>
       </c>
       <c r="C30" s="0">
-        <v>2465.19217585926</v>
+        <v>2465.19130007842</v>
       </c>
       <c r="D30" s="0">
-        <v>0.111042376717468</v>
+        <v>0.111042337268704</v>
       </c>
     </row>
     <row outlineLevel="0" r="31">
@@ -842,10 +842,10 @@
         <v>40692718.002</v>
       </c>
       <c r="C31" s="0">
-        <v>508.187131409644</v>
+        <v>508.161350653589</v>
       </c>
       <c r="D31" s="0">
-        <v>2.49768094323248E-02</v>
+        <v>2.49755423379983E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="32">
@@ -858,10 +858,10 @@
         <v>18764370.187</v>
       </c>
       <c r="C32" s="0">
-        <v>249.985244907066</v>
+        <v>249.983269913738</v>
       </c>
       <c r="D32" s="0">
-        <v>2.66446720476934E-02</v>
+        <v>2.66444615430714E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="33">
@@ -874,10 +874,10 @@
         <v>65039128.884</v>
       </c>
       <c r="C33" s="0">
-        <v>933.43284055604</v>
+        <v>933.38942808332</v>
       </c>
       <c r="D33" s="0">
-        <v>2.87037313252106E-02</v>
+        <v>2.87023963604451E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="34">
@@ -890,10 +890,10 @@
         <v>40853345.001</v>
       </c>
       <c r="C34" s="0">
-        <v>1342.73806852201</v>
+        <v>1342.73104450883</v>
       </c>
       <c r="D34" s="0">
-        <v>6.57345472440089E-02</v>
+        <v>6.57342033792319E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="35">
@@ -906,10 +906,10 @@
         <v>41832941.006</v>
       </c>
       <c r="C35" s="0">
-        <v>1055.65823213683</v>
+        <v>1055.65452444918</v>
       </c>
       <c r="D35" s="0">
-        <v>5.04701896041888E-02</v>
+        <v>5.04700123425588E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="36">
@@ -922,10 +922,10 @@
         <v>124473610.617</v>
       </c>
       <c r="C36" s="0">
-        <v>3289.61545460296</v>
+        <v>3289.5776725945</v>
       </c>
       <c r="D36" s="0">
-        <v>5.28564317897866E-02</v>
+        <v>5.28558247212157E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="37">
@@ -938,10 +938,10 @@
         <v>135802728.736</v>
       </c>
       <c r="C37" s="0">
-        <v>4751.17751565147</v>
+        <v>4751.05694326182</v>
       </c>
       <c r="D37" s="0">
-        <v>6.99717532905799E-02</v>
+        <v>6.99699775915087E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="38">
@@ -954,10 +954,10 @@
         <v>84634922.609</v>
       </c>
       <c r="C38" s="0">
-        <v>1145.03479518491</v>
+        <v>1144.99297015621</v>
       </c>
       <c r="D38" s="0">
-        <v>2.70582109580176E-02</v>
+        <v>2.70572225946467E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="39">
@@ -970,10 +970,10 @@
         <v>61254900.841</v>
       </c>
       <c r="C39" s="0">
-        <v>742.603908797989</v>
+        <v>742.603303365048</v>
       </c>
       <c r="D39" s="0">
-        <v>2.42463508585403E-02</v>
+        <v>0.024246331090883</v>
       </c>
     </row>
     <row outlineLevel="0" r="40">
@@ -986,10 +986,10 @@
         <v>239261130.761</v>
       </c>
       <c r="C40" s="0">
-        <v>4535.00448365747</v>
+        <v>4534.94599141405</v>
       </c>
       <c r="D40" s="0">
-        <v>3.79084096880535E-02</v>
+        <v>3.79079207474285E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="41">
@@ -1018,10 +1018,10 @@
         <v>7804400.21</v>
       </c>
       <c r="C42" s="0">
-        <v>151.577104965722</v>
+        <v>151.568542410447</v>
       </c>
       <c r="D42" s="0">
-        <v>3.88440112980116E-02</v>
+        <v>3.88418170088811E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="43">
@@ -1034,10 +1034,10 @@
         <v>98658089.209</v>
       </c>
       <c r="C43" s="0">
-        <v>2371.74510450447</v>
+        <v>2371.72877389775</v>
       </c>
       <c r="D43" s="0">
-        <v>4.80800940606118E-02</v>
+        <v>0.04807976300602</v>
       </c>
     </row>
     <row outlineLevel="0" r="44">
@@ -1050,10 +1050,10 @@
         <v>17900462.342</v>
       </c>
       <c r="C44" s="0">
-        <v>40.4139615804159</v>
+        <v>40.3840968992587</v>
       </c>
       <c r="D44" s="0">
-        <v>4.51540980431465E-03</v>
+        <v>4.5120730546166E-03</v>
       </c>
     </row>
     <row outlineLevel="0" r="45">
@@ -1066,10 +1066,10 @@
         <v>78032791.39</v>
       </c>
       <c r="C45" s="0">
-        <v>2212.11150389702</v>
+        <v>2212.04870286021</v>
       </c>
       <c r="D45" s="0">
-        <v>5.66969722469905E-02</v>
+        <v>0.056695362640678</v>
       </c>
     </row>
     <row outlineLevel="0" r="46">
@@ -1082,10 +1082,10 @@
         <v>521881132.673</v>
       </c>
       <c r="C46" s="0">
-        <v>12250.8913675252</v>
+        <v>12249.9035208392</v>
       </c>
       <c r="D46" s="0">
-        <v>4.69489720955342E-02</v>
+        <v>4.69451863802662E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="47">
@@ -1098,10 +1098,10 @@
         <v>39386042.997</v>
       </c>
       <c r="C47" s="0">
-        <v>1805.68807574896</v>
+        <v>1805.62911150598</v>
       </c>
       <c r="D47" s="0">
-        <v>9.16917739558906E-02</v>
+        <v>9.16887797864595E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="48">
@@ -1114,10 +1114,10 @@
         <v>89477324.859</v>
       </c>
       <c r="C48" s="0">
-        <v>1865.5709765427</v>
+        <v>1865.55815197244</v>
       </c>
       <c r="D48" s="0">
-        <v>4.16993015712641E-02</v>
+        <v>4.16990149160633E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="49">
@@ -1146,10 +1146,10 @@
         <v>116650629.994</v>
       </c>
       <c r="C50" s="0">
-        <v>1103.75548087203</v>
+        <v>1103.68257415845</v>
       </c>
       <c r="D50" s="0">
-        <v>1.89241237861948E-02</v>
+        <v>1.89228737849974E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="51">
@@ -1162,10 +1162,10 @@
         <v>61228765.961</v>
       </c>
       <c r="C51" s="0">
-        <v>1036.57187705787</v>
+        <v>1036.56632191194</v>
       </c>
       <c r="D51" s="0">
-        <v>3.38589831360679E-02</v>
+        <v>3.38588016806409E-02</v>
       </c>
     </row>
     <row outlineLevel="0" r="52">
@@ -1194,10 +1194,10 @@
         <v>46210977.449</v>
       </c>
       <c r="C53" s="0">
-        <v>1337.54202720269</v>
+        <v>1337.48246231747</v>
       </c>
       <c r="D53" s="0">
-        <v>5.78884975406047E-02</v>
+        <v>5.78859195866851E-02</v>
       </c>
     </row>
   </sheetData>
@@ -1486,13 +1486,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38083C74-77D1-44FA-B8A8-419E942AEE5F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DA27A723-84B1-4502-8E0C-5F086CEE08C5}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1104ACA0-50ED-4B60-ACE5-F0C67785AE73}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8081564D-AD85-4212-9067-F3D00CFA052E}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DD397F47-8914-4322-B35C-BAF7E9ADE317}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C3FEFFBA-1B49-4ED7-A1E1-573AFE3B172A}"/>
 </file>
</xml_diff>